<commit_message>
Add DLL for Data acquisition card
</commit_message>
<xml_diff>
--- a/TestInput.xlsx
+++ b/TestInput.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lijiangwei\Desktop\File\Auto_Test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C56ABC84-D80C-4363-8CE2-C109DD5E9104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{224443DE-B9D8-4093-A62A-1B065818266E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="24196" windowHeight="14476" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2348" yWindow="3083" windowWidth="17999" windowHeight="10432" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IC" sheetId="6" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="71">
   <si>
     <t>温度测试</t>
   </si>
@@ -279,6 +279,10 @@
   </si>
   <si>
     <t>TCPIP::192.168.18.100::INSTR</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>FIFO_Single_Test</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1177,7 +1181,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet6"/>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="36.59765625" customWidth="1"/>
@@ -1326,10 +1330,10 @@
     </row>
     <row r="7" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A7" s="10" t="s">
-        <v>32</v>
+        <v>70</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -1344,7 +1348,7 @@
     </row>
     <row r="8" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A8" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B8" s="9" t="s">
         <v>2</v>
@@ -1361,8 +1365,8 @@
       <c r="L8" s="7"/>
     </row>
     <row r="9" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A9" s="11" t="s">
-        <v>35</v>
+      <c r="A9" s="10" t="s">
+        <v>33</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>2</v>
@@ -1380,7 +1384,7 @@
     </row>
     <row r="10" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A10" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B10" s="9" t="s">
         <v>2</v>
@@ -1398,7 +1402,7 @@
     </row>
     <row r="11" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A11" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B11" s="9" t="s">
         <v>2</v>
@@ -1416,7 +1420,7 @@
     </row>
     <row r="12" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A12" s="11" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B12" s="9" t="s">
         <v>2</v>
@@ -1434,7 +1438,7 @@
     </row>
     <row r="13" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A13" s="11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B13" s="9" t="s">
         <v>2</v>
@@ -1452,21 +1456,39 @@
     </row>
     <row r="14" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A14" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="7"/>
+    </row>
+    <row r="15" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A15" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="B14" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="8"/>
-      <c r="J14" s="8"/>
-      <c r="K14" s="8"/>
-      <c r="L14" s="8"/>
+      <c r="B15" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1474,7 +1496,7 @@
     <mergeCell ref="C1:L1"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="B3:B14">
+  <conditionalFormatting sqref="B3:B15">
     <cfRule type="cellIs" dxfId="1" priority="7" operator="equal">
       <formula>"是"</formula>
     </cfRule>
@@ -1486,7 +1508,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L3" xr:uid="{4CCF8D95-9DCF-49A9-AD1F-1E411B1BC529}">
       <formula1>"Normal,5%,3%,All"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B14" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B15" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"是,否"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
add report,dll,and 34461A driver
</commit_message>
<xml_diff>
--- a/TestInput.xlsx
+++ b/TestInput.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lijiangwei\Desktop\File\Auto_Test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{224443DE-B9D8-4093-A62A-1B065818266E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8F3623B-9A68-4750-843F-E2D428062446}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2348" yWindow="3083" windowWidth="17999" windowHeight="10432" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2348" yWindow="3083" windowWidth="17999" windowHeight="10432" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IC" sheetId="6" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="71">
   <si>
     <t>温度测试</t>
   </si>
@@ -77,212 +77,221 @@
     <t>Power</t>
   </si>
   <si>
-    <t>IT6932A</t>
-  </si>
-  <si>
-    <t>USB0::0x2EC7::0x6900::800063020757810029::0::INSTR</t>
-  </si>
-  <si>
     <t>LOAD</t>
   </si>
   <si>
     <t>Eload</t>
   </si>
   <si>
-    <t>FT6301A</t>
+    <t>Chamber</t>
+  </si>
+  <si>
+    <t>ASRL2::INSTR</t>
+  </si>
+  <si>
+    <t>OSC</t>
+  </si>
+  <si>
+    <t>TCPIP0::LCRY4501N30096::inst0::INSTR</t>
+  </si>
+  <si>
+    <t>Tektronic</t>
+  </si>
+  <si>
+    <t>USB0::0x0699::0x052C::C034040::0::INSTR</t>
+  </si>
+  <si>
+    <t>Keysight</t>
+  </si>
+  <si>
+    <t>USB0::0x2A8D::0x1764::MY62510027::0::INSTR</t>
+  </si>
+  <si>
+    <t>Current</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ADC1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ADC2</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ADC3</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Vcore1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Vcore2</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Vcore3</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Vcore4</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Freq</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>VStart</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>VStop</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>VStep</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ADC4</t>
+  </si>
+  <si>
+    <t>ADC5</t>
+  </si>
+  <si>
+    <t>ADC6</t>
+  </si>
+  <si>
+    <t>FDev</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>参数</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>OSC</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>否</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>RohdeSchwarz</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Lecroy</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>COM</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MCU</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SerialPort</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>UR_Test</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>I2C_Test</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>QSPI_Test</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SPI_Test</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>CHA</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>KC</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>/</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>测试IC</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>BASE</t>
+  </si>
+  <si>
+    <t>TCPIP::192.168.18.100::INSTR</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>FIFO_Single_Test</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Trigger_Test</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ripple_Test</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>RMS_Test</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>34461A</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>USB0::0x2A8D::0x1301::MY64022314::INSTR</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DMM</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ASRL7::INSTR</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>USB0::0x0A69::0x0879::63210AL01706::INSTR</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>VCORE</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>Multimeter</t>
-  </si>
-  <si>
-    <t>I_M</t>
-  </si>
-  <si>
-    <t>34465A</t>
-  </si>
-  <si>
-    <t>USB0::0x2A8D::0x0101::MY60060781::0::INSTR</t>
-  </si>
-  <si>
-    <t>V_M</t>
-  </si>
-  <si>
-    <t>USB0::0x2A8D::0x0101::MY60005730::0::INSTR</t>
-  </si>
-  <si>
-    <t>Chamber</t>
-  </si>
-  <si>
-    <t>ASRL2::INSTR</t>
-  </si>
-  <si>
-    <t>OSC</t>
-  </si>
-  <si>
-    <t>TCPIP0::LCRY4501N30096::inst0::INSTR</t>
-  </si>
-  <si>
-    <t>Tektronic</t>
-  </si>
-  <si>
-    <t>USB0::0x0699::0x052C::C034040::0::INSTR</t>
-  </si>
-  <si>
-    <t>Keysight</t>
-  </si>
-  <si>
-    <t>USB0::0x2A8D::0x1764::MY62510027::0::INSTR</t>
-  </si>
-  <si>
-    <t>Ripple</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>RMS</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Current</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>ADC1</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>ADC2</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>ADC3</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Vcore1</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Vcore2</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Vcore3</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Vcore4</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Freq</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>VStart</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>VStop</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>VStep</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>ADC4</t>
-  </si>
-  <si>
-    <t>ADC5</t>
-  </si>
-  <si>
-    <t>ADC6</t>
-  </si>
-  <si>
-    <t>FDev</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>参数</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>OSC</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>否</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>RohdeSchwarz</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Lecroy</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>COM</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>MCU</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>ASRL5::INSTR</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>SerialPort</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>UR_Test</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>I2C_Test</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>QSPI_Test</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>SPI_Test</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>PWVCORE</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>CHA</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>KC</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>/</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>测试IC</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>BASE</t>
-  </si>
-  <si>
-    <t>TCPIP::192.168.18.100::INSTR</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>FIFO_Single_Test</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>PS9080</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>63200A</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ASRL6::INSTR</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -484,7 +493,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -518,6 +527,8 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -861,7 +872,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="18" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>0</v>
@@ -872,7 +883,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" s="17" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>2</v>
@@ -942,7 +953,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="2" width="11.46484375" customWidth="1"/>
@@ -970,50 +981,50 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D2" s="15" t="s">
-        <v>57</v>
+        <v>14</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>65</v>
       </c>
       <c r="E2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A3" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>21</v>
+    <row r="3" spans="1:5" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>62</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="2" t="s">
-        <v>22</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A4" s="15" t="s">
+        <v>66</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>23</v>
+        <v>12</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>64</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>2</v>
@@ -1021,33 +1032,33 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A5" s="15" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>52</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A6" s="15" t="s">
-        <v>64</v>
+      <c r="A6" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>2</v>
@@ -1055,16 +1066,16 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>54</v>
+        <v>17</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>19</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>2</v>
@@ -1072,16 +1083,16 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>26</v>
+        <v>17</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>40</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>2</v>
@@ -1089,75 +1100,58 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>30</v>
+        <v>40</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>42</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>2</v>
+        <v>22</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>56</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>52</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A11" s="2" t="s">
-        <v>26</v>
+      <c r="A11" s="15" t="s">
+        <v>45</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A12" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="B12" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="C12" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="D12" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="E12" s="15" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="E2:E12">
+  <conditionalFormatting sqref="E2:E11">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"是"</formula>
     </cfRule>
@@ -1169,7 +1163,7 @@
     <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"是,否"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3:E12" xr:uid="{00000000-0002-0000-0200-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3:E11" xr:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>"是,否"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1181,7 +1175,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet6"/>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="36.59765625" customWidth="1"/>
@@ -1195,22 +1189,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="23"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
+      <c r="L1" s="25"/>
     </row>
     <row r="2" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A2" s="13" t="s">
@@ -1220,39 +1214,39 @@
         <v>5</v>
       </c>
       <c r="C2" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="G2" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="H2" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="I2" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="J2" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="K2" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="L2" s="14" t="s">
         <v>38</v>
-      </c>
-      <c r="E2" s="14" t="s">
-        <v>39</v>
-      </c>
-      <c r="F2" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="G2" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="H2" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="I2" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="J2" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="K2" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="L2" s="14" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A3" s="10" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>6</v>
@@ -1260,10 +1254,10 @@
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
       <c r="E3" s="16" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
@@ -1276,10 +1270,10 @@
     </row>
     <row r="4" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A4" s="10" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -1294,7 +1288,7 @@
     </row>
     <row r="5" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A5" s="10" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>2</v>
@@ -1312,7 +1306,7 @@
     </row>
     <row r="6" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A6" s="10" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>2</v>
@@ -1330,10 +1324,10 @@
     </row>
     <row r="7" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A7" s="10" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -1348,7 +1342,7 @@
     </row>
     <row r="8" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A8" s="10" t="s">
-        <v>32</v>
+        <v>59</v>
       </c>
       <c r="B8" s="9" t="s">
         <v>2</v>
@@ -1366,7 +1360,7 @@
     </row>
     <row r="9" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A9" s="10" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>2</v>
@@ -1383,8 +1377,8 @@
       <c r="L9" s="7"/>
     </row>
     <row r="10" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="11" t="s">
-        <v>35</v>
+      <c r="A10" s="10" t="s">
+        <v>58</v>
       </c>
       <c r="B10" s="9" t="s">
         <v>2</v>
@@ -1402,7 +1396,7 @@
     </row>
     <row r="11" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A11" s="11" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="B11" s="9" t="s">
         <v>2</v>
@@ -1420,7 +1414,7 @@
     </row>
     <row r="12" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A12" s="11" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="B12" s="9" t="s">
         <v>2</v>
@@ -1438,7 +1432,7 @@
     </row>
     <row r="13" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A13" s="11" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="B13" s="9" t="s">
         <v>2</v>
@@ -1456,7 +1450,7 @@
     </row>
     <row r="14" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A14" s="11" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="B14" s="9" t="s">
         <v>2</v>
@@ -1474,21 +1468,39 @@
     </row>
     <row r="15" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A15" s="11" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="B15" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="8"/>
-      <c r="I15" s="8"/>
-      <c r="J15" s="8"/>
-      <c r="K15" s="8"/>
-      <c r="L15" s="8"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
+      <c r="J15" s="7"/>
+      <c r="K15" s="7"/>
+      <c r="L15" s="7"/>
+    </row>
+    <row r="16" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A16" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="8"/>
+      <c r="L16" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1496,7 +1508,7 @@
     <mergeCell ref="C1:L1"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="B3:B15">
+  <conditionalFormatting sqref="B3:B16">
     <cfRule type="cellIs" dxfId="1" priority="7" operator="equal">
       <formula>"是"</formula>
     </cfRule>
@@ -1508,7 +1520,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L3" xr:uid="{4CCF8D95-9DCF-49A9-AD1F-1E411B1BC529}">
       <formula1>"Normal,5%,3%,All"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B15" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B16" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"是,否"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Create a new branch
</commit_message>
<xml_diff>
--- a/TestInput.xlsx
+++ b/TestInput.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lijiangwei\Desktop\File\Auto_Test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8F3623B-9A68-4750-843F-E2D428062446}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4C5EE92-3DC4-4770-8D4D-B22B668D3E71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2348" yWindow="3083" windowWidth="17999" windowHeight="10432" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="72">
   <si>
     <t>温度测试</t>
   </si>
@@ -263,10 +263,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>DMM</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>ASRL7::INSTR</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -292,6 +288,14 @@
   </si>
   <si>
     <t>ASRL6::INSTR</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>VDMM</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>IDMM</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -953,7 +957,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="2" width="11.46484375" customWidth="1"/>
@@ -987,10 +991,10 @@
         <v>14</v>
       </c>
       <c r="C2" s="20" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E2" t="s">
         <v>2</v>
@@ -998,10 +1002,10 @@
     </row>
     <row r="3" spans="1:5" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="15" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C3" s="15" t="s">
         <v>61</v>
@@ -1013,18 +1017,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:5" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="C4" s="15" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>2</v>
@@ -1032,33 +1036,33 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A5" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A6" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C6" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>18</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>2</v>
@@ -1071,11 +1075,11 @@
       <c r="B7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>19</v>
+      <c r="C7" s="15" t="s">
+        <v>43</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>2</v>
@@ -1085,14 +1089,14 @@
       <c r="A8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="15" t="s">
-        <v>40</v>
+      <c r="B8" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>2</v>
@@ -1105,14 +1109,14 @@
       <c r="B9" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="15" t="s">
-        <v>42</v>
+      <c r="C9" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E9" s="15" t="s">
-        <v>41</v>
+      <c r="E9" s="2" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.4">
@@ -1125,33 +1129,50 @@
       <c r="C10" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="D11" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="E10" s="15" t="s">
+      <c r="E11" s="15" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A11" s="15" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A12" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B12" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C12" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="D11" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="E11" s="15" t="s">
+      <c r="D12" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="E12" s="15" t="s">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="E2:E11">
+  <conditionalFormatting sqref="E2:E12">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"是"</formula>
     </cfRule>
@@ -1163,7 +1184,7 @@
     <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"是,否"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3:E11" xr:uid="{00000000-0002-0000-0200-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3:E12" xr:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>"是,否"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add eload 63210A driver and ps9080 driver,translate comment in to english
</commit_message>
<xml_diff>
--- a/TestInput.xlsx
+++ b/TestInput.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lijiangwei\Desktop\File\Auto_Test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4C5EE92-3DC4-4770-8D4D-B22B668D3E71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EC43F93-D462-41BA-B2D2-1A06CC941EFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2348" yWindow="3083" windowWidth="17999" windowHeight="10432" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -74,228 +74,230 @@
     <t>是否初始化</t>
   </si>
   <si>
-    <t>Power</t>
-  </si>
-  <si>
     <t>LOAD</t>
   </si>
   <si>
+    <t>Chamber</t>
+  </si>
+  <si>
+    <t>ASRL2::INSTR</t>
+  </si>
+  <si>
+    <t>OSC</t>
+  </si>
+  <si>
+    <t>TCPIP0::LCRY4501N30096::inst0::INSTR</t>
+  </si>
+  <si>
+    <t>Tektronic</t>
+  </si>
+  <si>
+    <t>USB0::0x0699::0x052C::C034040::0::INSTR</t>
+  </si>
+  <si>
+    <t>Keysight</t>
+  </si>
+  <si>
+    <t>USB0::0x2A8D::0x1764::MY62510027::0::INSTR</t>
+  </si>
+  <si>
+    <t>Current</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ADC1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ADC2</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ADC3</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Vcore1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Vcore2</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Vcore3</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Vcore4</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Freq</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>VStart</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>VStop</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>VStep</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ADC4</t>
+  </si>
+  <si>
+    <t>ADC5</t>
+  </si>
+  <si>
+    <t>ADC6</t>
+  </si>
+  <si>
+    <t>FDev</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>参数</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>OSC</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>否</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>RohdeSchwarz</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Lecroy</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>COM</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MCU</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SerialPort</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>UR_Test</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>I2C_Test</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>QSPI_Test</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SPI_Test</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>CHA</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>KC</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>/</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>测试IC</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>BASE</t>
+  </si>
+  <si>
+    <t>TCPIP::192.168.18.100::INSTR</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>FIFO_Single_Test</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Trigger_Test</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ripple_Test</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>RMS_Test</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>34461A</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>USB0::0x2A8D::0x1301::MY64022314::INSTR</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ASRL7::INSTR</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>USB0::0x0A69::0x0879::63210AL01706::INSTR</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Multimeter</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>PS9080</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>63200A</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ASRL6::INSTR</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>VDMM</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>IDMM</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>Eload</t>
-  </si>
-  <si>
-    <t>Chamber</t>
-  </si>
-  <si>
-    <t>ASRL2::INSTR</t>
-  </si>
-  <si>
-    <t>OSC</t>
-  </si>
-  <si>
-    <t>TCPIP0::LCRY4501N30096::inst0::INSTR</t>
-  </si>
-  <si>
-    <t>Tektronic</t>
-  </si>
-  <si>
-    <t>USB0::0x0699::0x052C::C034040::0::INSTR</t>
-  </si>
-  <si>
-    <t>Keysight</t>
-  </si>
-  <si>
-    <t>USB0::0x2A8D::0x1764::MY62510027::0::INSTR</t>
-  </si>
-  <si>
-    <t>Current</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>ADC1</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>ADC2</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>ADC3</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Vcore1</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Vcore2</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Vcore3</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Vcore4</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Freq</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>VStart</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>VStop</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>VStep</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>ADC4</t>
-  </si>
-  <si>
-    <t>ADC5</t>
-  </si>
-  <si>
-    <t>ADC6</t>
-  </si>
-  <si>
-    <t>FDev</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>参数</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>OSC</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>否</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>RohdeSchwarz</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Lecroy</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>COM</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>MCU</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>SerialPort</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>UR_Test</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>I2C_Test</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>QSPI_Test</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>SPI_Test</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>CHA</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>KC</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>/</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>测试IC</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>BASE</t>
-  </si>
-  <si>
-    <t>TCPIP::192.168.18.100::INSTR</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>FIFO_Single_Test</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Trigger_Test</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Ripple_Test</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>RMS_Test</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>34461A</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>USB0::0x2A8D::0x1301::MY64022314::INSTR</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>ASRL7::INSTR</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>USB0::0x0A69::0x0879::63210AL01706::INSTR</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>VCORE</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Multimeter</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>PS9080</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>63200A</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>ASRL6::INSTR</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>VDMM</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>IDMM</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>PSU</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>POW</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -876,7 +878,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="18" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>0</v>
@@ -887,7 +889,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" s="17" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>2</v>
@@ -985,16 +987,16 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>69</v>
       </c>
       <c r="C2" s="20" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E2" t="s">
         <v>2</v>
@@ -1002,16 +1004,16 @@
     </row>
     <row r="3" spans="1:5" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>6</v>
@@ -1019,16 +1021,16 @@
     </row>
     <row r="4" spans="1:5" ht="13.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="15" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>2</v>
@@ -1036,16 +1038,16 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A5" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>12</v>
+        <v>71</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>70</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>2</v>
@@ -1053,16 +1055,16 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A6" s="15" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>2</v>
@@ -1070,16 +1072,16 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>2</v>
@@ -1087,16 +1089,16 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="D8" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>2</v>
@@ -1104,16 +1106,16 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>2</v>
@@ -1121,33 +1123,33 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B10" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="15" t="s">
-        <v>42</v>
-      </c>
       <c r="D10" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B11" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="C11" s="15" t="s">
-        <v>42</v>
-      </c>
       <c r="D11" s="15" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E11" s="15" t="s">
         <v>6</v>
@@ -1155,16 +1157,16 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A12" s="15" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B12" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="C12" s="15" t="s">
-        <v>46</v>
-      </c>
       <c r="D12" s="15" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E12" s="15" t="s">
         <v>2</v>
@@ -1215,7 +1217,7 @@
       </c>
       <c r="B1" s="22"/>
       <c r="C1" s="23" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D1" s="24"/>
       <c r="E1" s="24"/>
@@ -1235,39 +1237,39 @@
         <v>5</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D2" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="G2" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="F2" s="14" t="s">
+      <c r="H2" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="I2" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="H2" s="14" t="s">
+      <c r="J2" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="I2" s="14" t="s">
+      <c r="K2" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="J2" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="K2" s="14" t="s">
-        <v>34</v>
-      </c>
       <c r="L2" s="14" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A3" s="10" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>6</v>
@@ -1275,10 +1277,10 @@
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
       <c r="E3" s="16" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
@@ -1291,7 +1293,7 @@
     </row>
     <row r="4" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A4" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B4" s="9" t="s">
         <v>2</v>
@@ -1309,7 +1311,7 @@
     </row>
     <row r="5" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A5" s="10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>2</v>
@@ -1327,7 +1329,7 @@
     </row>
     <row r="6" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A6" s="10" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>2</v>
@@ -1345,7 +1347,7 @@
     </row>
     <row r="7" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A7" s="10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>2</v>
@@ -1363,7 +1365,7 @@
     </row>
     <row r="8" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A8" s="10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B8" s="9" t="s">
         <v>2</v>
@@ -1381,7 +1383,7 @@
     </row>
     <row r="9" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A9" s="10" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>2</v>
@@ -1399,7 +1401,7 @@
     </row>
     <row r="10" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A10" s="10" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B10" s="9" t="s">
         <v>2</v>
@@ -1417,7 +1419,7 @@
     </row>
     <row r="11" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A11" s="11" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B11" s="9" t="s">
         <v>2</v>
@@ -1435,7 +1437,7 @@
     </row>
     <row r="12" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A12" s="11" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B12" s="9" t="s">
         <v>2</v>
@@ -1453,7 +1455,7 @@
     </row>
     <row r="13" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A13" s="11" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B13" s="9" t="s">
         <v>2</v>
@@ -1471,7 +1473,7 @@
     </row>
     <row r="14" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A14" s="11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B14" s="9" t="s">
         <v>2</v>
@@ -1489,7 +1491,7 @@
     </row>
     <row r="15" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A15" s="11" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B15" s="9" t="s">
         <v>2</v>
@@ -1507,7 +1509,7 @@
     </row>
     <row r="16" spans="1:12" ht="14.25" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A16" s="11" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B16" s="9" t="s">
         <v>2</v>

</xml_diff>

<commit_message>
Add keysight53250 and DAQ973A driver
</commit_message>
<xml_diff>
--- a/TestInput.xlsx
+++ b/TestInput.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lijiangwei\Desktop\File\Auto_Test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EC43F93-D462-41BA-B2D2-1A06CC941EFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C3ABF96-728D-45F4-9EBE-187B5C7E9055}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2348" yWindow="3083" windowWidth="17999" windowHeight="10432" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="24196" windowHeight="14476" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IC" sheetId="6" r:id="rId1"/>
@@ -1272,7 +1272,7 @@
         <v>45</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
@@ -1296,7 +1296,7 @@
         <v>46</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>

</xml_diff>